<commit_message>
Clean-up in syntax_helper, finished syntax_helper::parse_line
</commit_message>
<xml_diff>
--- a/Xis16 Spreadsheet.xlsx
+++ b/Xis16 Spreadsheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
   <si>
     <t xml:space="preserve">Byte 1</t>
   </si>
@@ -202,6 +202,15 @@
   </si>
   <si>
     <t xml:space="preserve">C &lt;- A &lt;&lt; 1 (physical shift)</t>
+  </si>
+  <si>
+    <t>SHF</t>
+  </si>
+  <si>
+    <t>Shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C &lt;- A &gt;&gt; B </t>
   </si>
   <si>
     <t>LDI</t>
@@ -436,7 +445,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -451,12 +460,6 @@
     <font>
       <sz val="9.000000"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="17">
@@ -557,7 +560,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="5">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -584,7 +587,7 @@
       <left style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </left>
-      <right/>
+      <right style="none"/>
       <top style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </top>
@@ -594,8 +597,8 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </top>
@@ -605,7 +608,7 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left/>
+      <left style="none"/>
       <right style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </right>
@@ -617,48 +620,11 @@
       </bottom>
       <diagonal style="none"/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -675,9 +641,6 @@
     <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -688,7 +651,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -705,17 +668,32 @@
     <xf fontId="1" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="2" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -729,9 +707,6 @@
     <xf fontId="2" fillId="14" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="1" fillId="15" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -744,29 +719,23 @@
     <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="5" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="5" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="3" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="16" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1480,7 +1449,7 @@
       <c r="AB4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AC4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="AD4" s="1"/>
@@ -1497,10 +1466,10 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2"/>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="5">
@@ -1518,29 +1487,29 @@
       <c r="H5" s="2">
         <v>0</v>
       </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8"/>
-      <c r="Y5" s="8"/>
-      <c r="Z5" s="8"/>
-      <c r="AA5" s="8"/>
-      <c r="AB5" s="9" t="s">
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="7"/>
+      <c r="AB5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC5" s="10" t="s">
+      <c r="AC5" s="9" t="s">
         <v>12</v>
       </c>
       <c r="AD5" s="1"/>
@@ -1555,10 +1524,10 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2"/>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="2">
@@ -1573,32 +1542,32 @@
       <c r="G6" s="2">
         <v>0</v>
       </c>
-      <c r="H6" s="11">
-        <v>1</v>
-      </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="8"/>
-      <c r="W6" s="8"/>
-      <c r="X6" s="8"/>
-      <c r="Y6" s="8"/>
-      <c r="Z6" s="8"/>
-      <c r="AA6" s="8"/>
-      <c r="AB6" s="9" t="s">
+      <c r="H6" s="10">
+        <v>1</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="7"/>
+      <c r="V6" s="7"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="7"/>
+      <c r="AB6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC6" s="10" t="s">
+      <c r="AC6" s="9" t="s">
         <v>15</v>
       </c>
       <c r="AD6" s="1"/>
@@ -1613,10 +1582,10 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2"/>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="11" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="2">
@@ -1628,7 +1597,7 @@
       <c r="F7" s="2">
         <v>0</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <v>1</v>
       </c>
       <c r="H7" s="2">
@@ -1649,20 +1618,20 @@
       </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
-      <c r="V7" s="8"/>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8"/>
-      <c r="Y7" s="8"/>
-      <c r="Z7" s="8"/>
-      <c r="AA7" s="8"/>
-      <c r="AB7" s="13" t="s">
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC7" s="6" t="s">
+      <c r="AC7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="AD7" s="1"/>
@@ -1677,10 +1646,10 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2"/>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="2">
@@ -1692,10 +1661,10 @@
       <c r="F8" s="2">
         <v>0</v>
       </c>
-      <c r="G8" s="11">
-        <v>1</v>
-      </c>
-      <c r="H8" s="11">
+      <c r="G8" s="10">
+        <v>1</v>
+      </c>
+      <c r="H8" s="10">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -1713,20 +1682,20 @@
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
-      <c r="V8" s="8"/>
-      <c r="W8" s="8"/>
-      <c r="X8" s="8"/>
-      <c r="Y8" s="8"/>
-      <c r="Z8" s="8"/>
-      <c r="AA8" s="8"/>
-      <c r="AB8" s="13" t="s">
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC8" s="6" t="s">
+      <c r="AC8" s="3" t="s">
         <v>25</v>
       </c>
       <c r="AD8" s="1"/>
@@ -1741,10 +1710,10 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2"/>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="13" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="2">
@@ -1753,7 +1722,7 @@
       <c r="E9" s="2">
         <v>0</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <v>1</v>
       </c>
       <c r="G9" s="2">
@@ -1777,20 +1746,20 @@
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
-      <c r="R9" s="8"/>
-      <c r="S9" s="8"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="8"/>
-      <c r="V9" s="8"/>
-      <c r="W9" s="8"/>
-      <c r="X9" s="8"/>
-      <c r="Y9" s="8"/>
-      <c r="Z9" s="8"/>
-      <c r="AA9" s="8"/>
-      <c r="AB9" s="13" t="s">
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="7"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="7"/>
+      <c r="AB9" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC9" s="6" t="s">
+      <c r="AC9" s="3" t="s">
         <v>28</v>
       </c>
       <c r="AD9" s="1"/>
@@ -1805,10 +1774,10 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2"/>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="13" t="s">
         <v>30</v>
       </c>
       <c r="D10" s="2">
@@ -1817,13 +1786,13 @@
       <c r="E10" s="2">
         <v>0</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="10">
         <v>1</v>
       </c>
       <c r="G10" s="2">
         <v>0</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="14">
         <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -1841,20 +1810,20 @@
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8"/>
-      <c r="AA10" s="8"/>
-      <c r="AB10" s="13" t="s">
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
+      <c r="V10" s="7"/>
+      <c r="W10" s="7"/>
+      <c r="X10" s="7"/>
+      <c r="Y10" s="7"/>
+      <c r="Z10" s="7"/>
+      <c r="AA10" s="7"/>
+      <c r="AB10" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC10" s="6" t="s">
+      <c r="AC10" s="3" t="s">
         <v>31</v>
       </c>
       <c r="AD10" s="1"/>
@@ -1869,10 +1838,10 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2"/>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="13" t="s">
         <v>33</v>
       </c>
       <c r="D11" s="2">
@@ -1881,10 +1850,10 @@
       <c r="E11" s="2">
         <v>0</v>
       </c>
-      <c r="F11" s="11">
-        <v>1</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="10">
+        <v>1</v>
+      </c>
+      <c r="G11" s="10">
         <v>1</v>
       </c>
       <c r="H11" s="2">
@@ -1905,20 +1874,20 @@
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
-      <c r="R11" s="8"/>
-      <c r="S11" s="8"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="8"/>
-      <c r="W11" s="8"/>
-      <c r="X11" s="8"/>
-      <c r="Y11" s="8"/>
-      <c r="Z11" s="8"/>
-      <c r="AA11" s="8"/>
-      <c r="AB11" s="13" t="s">
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7"/>
+      <c r="AA11" s="7"/>
+      <c r="AB11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC11" s="6" t="s">
+      <c r="AC11" s="3" t="s">
         <v>34</v>
       </c>
       <c r="AD11" s="1"/>
@@ -1933,10 +1902,10 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2"/>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>36</v>
       </c>
       <c r="D12" s="2">
@@ -1945,13 +1914,13 @@
       <c r="E12" s="2">
         <v>0</v>
       </c>
-      <c r="F12" s="11">
-        <v>1</v>
-      </c>
-      <c r="G12" s="11">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11">
+      <c r="F12" s="10">
+        <v>1</v>
+      </c>
+      <c r="G12" s="10">
+        <v>1</v>
+      </c>
+      <c r="H12" s="10">
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
@@ -1969,20 +1938,20 @@
       </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8"/>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="8"/>
-      <c r="AA12" s="8"/>
-      <c r="AB12" s="13" t="s">
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="7"/>
+      <c r="AB12" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC12" s="6" t="s">
+      <c r="AC12" s="3" t="s">
         <v>37</v>
       </c>
       <c r="AI12" s="1"/>
@@ -1998,16 +1967,16 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>39</v>
       </c>
       <c r="D13" s="2">
         <v>0</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="10">
         <v>1</v>
       </c>
       <c r="F13" s="2">
@@ -2034,20 +2003,20 @@
       </c>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
-      <c r="R13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
-      <c r="W13" s="8"/>
-      <c r="X13" s="8"/>
-      <c r="Y13" s="8"/>
-      <c r="Z13" s="8"/>
-      <c r="AA13" s="8"/>
-      <c r="AB13" s="13" t="s">
+      <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
+      <c r="X13" s="7"/>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="7"/>
+      <c r="AA13" s="7"/>
+      <c r="AB13" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC13" s="6" t="s">
+      <c r="AC13" s="3" t="s">
         <v>40</v>
       </c>
       <c r="AD13" s="1"/>
@@ -2063,16 +2032,16 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="2">
         <v>0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>1</v>
       </c>
       <c r="F14" s="2">
@@ -2081,7 +2050,7 @@
       <c r="G14" s="2">
         <v>0</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <v>1</v>
       </c>
       <c r="I14" s="1" t="s">
@@ -2099,20 +2068,20 @@
       </c>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
-      <c r="R14" s="8"/>
-      <c r="S14" s="8"/>
-      <c r="T14" s="8"/>
-      <c r="U14" s="8"/>
-      <c r="V14" s="8"/>
-      <c r="W14" s="8"/>
-      <c r="X14" s="8"/>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="8"/>
-      <c r="AA14" s="8"/>
-      <c r="AB14" s="13" t="s">
+      <c r="R14" s="7"/>
+      <c r="S14" s="7"/>
+      <c r="T14" s="7"/>
+      <c r="U14" s="7"/>
+      <c r="V14" s="7"/>
+      <c r="W14" s="7"/>
+      <c r="X14" s="7"/>
+      <c r="Y14" s="7"/>
+      <c r="Z14" s="7"/>
+      <c r="AA14" s="7"/>
+      <c r="AB14" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC14" s="6" t="s">
+      <c r="AC14" s="3" t="s">
         <v>43</v>
       </c>
       <c r="AD14" s="1"/>
@@ -2128,22 +2097,22 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2"/>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>45</v>
       </c>
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="10">
         <v>1</v>
       </c>
       <c r="F15" s="2">
         <v>0</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>1</v>
       </c>
       <c r="H15" s="2">
@@ -2164,20 +2133,20 @@
       </c>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
-      <c r="R15" s="8"/>
-      <c r="S15" s="8"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="8"/>
-      <c r="V15" s="8"/>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
-      <c r="Y15" s="8"/>
-      <c r="Z15" s="8"/>
-      <c r="AA15" s="8"/>
-      <c r="AB15" s="13" t="s">
+      <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
+      <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
+      <c r="Z15" s="7"/>
+      <c r="AA15" s="7"/>
+      <c r="AB15" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC15" s="6" t="s">
+      <c r="AC15" s="3" t="s">
         <v>46</v>
       </c>
       <c r="AD15" s="1"/>
@@ -2193,25 +2162,25 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2"/>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="11" t="s">
         <v>48</v>
       </c>
       <c r="D16" s="2">
         <v>0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="10">
         <v>1</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
       </c>
-      <c r="G16" s="11">
-        <v>1</v>
-      </c>
-      <c r="H16" s="11">
+      <c r="G16" s="10">
+        <v>1</v>
+      </c>
+      <c r="H16" s="10">
         <v>1</v>
       </c>
       <c r="I16" s="1" t="s">
@@ -2229,20 +2198,20 @@
       </c>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
-      <c r="R16" s="8"/>
-      <c r="S16" s="8"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="8"/>
-      <c r="V16" s="8"/>
-      <c r="W16" s="8"/>
-      <c r="X16" s="8"/>
-      <c r="Y16" s="8"/>
-      <c r="Z16" s="8"/>
-      <c r="AA16" s="8"/>
-      <c r="AB16" s="13" t="s">
+      <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
+      <c r="T16" s="7"/>
+      <c r="U16" s="7"/>
+      <c r="V16" s="7"/>
+      <c r="W16" s="7"/>
+      <c r="X16" s="7"/>
+      <c r="Y16" s="7"/>
+      <c r="Z16" s="7"/>
+      <c r="AA16" s="7"/>
+      <c r="AB16" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC16" s="6" t="s">
+      <c r="AC16" s="3" t="s">
         <v>49</v>
       </c>
       <c r="AD16" s="1"/>
@@ -2258,19 +2227,19 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2"/>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="11" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="2">
         <v>0</v>
       </c>
-      <c r="E17" s="11">
-        <v>1</v>
-      </c>
-      <c r="F17" s="11">
+      <c r="E17" s="10">
+        <v>1</v>
+      </c>
+      <c r="F17" s="10">
         <v>1</v>
       </c>
       <c r="G17" s="2">
@@ -2294,20 +2263,20 @@
       </c>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="8"/>
-      <c r="Z17" s="8"/>
-      <c r="AA17" s="8"/>
-      <c r="AB17" s="13" t="s">
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
+      <c r="Z17" s="7"/>
+      <c r="AA17" s="7"/>
+      <c r="AB17" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC17" s="6" t="s">
+      <c r="AC17" s="3" t="s">
         <v>52</v>
       </c>
       <c r="AD17" s="1"/>
@@ -2323,25 +2292,25 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2"/>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="11" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
       </c>
-      <c r="E18" s="11">
-        <v>1</v>
-      </c>
-      <c r="F18" s="11">
+      <c r="E18" s="10">
+        <v>1</v>
+      </c>
+      <c r="F18" s="10">
         <v>1</v>
       </c>
       <c r="G18" s="2">
         <v>0</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="10">
         <v>1</v>
       </c>
       <c r="I18" s="1" t="s">
@@ -2354,23 +2323,23 @@
       </c>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8"/>
-      <c r="S18" s="8"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="8"/>
-      <c r="V18" s="8"/>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
-      <c r="Y18" s="8"/>
-      <c r="Z18" s="8"/>
-      <c r="AA18" s="8"/>
-      <c r="AB18" s="13" t="s">
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
+      <c r="Z18" s="7"/>
+      <c r="AA18" s="7"/>
+      <c r="AB18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC18" s="6" t="s">
+      <c r="AC18" s="3" t="s">
         <v>55</v>
       </c>
       <c r="AD18" s="1"/>
@@ -2386,22 +2355,22 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2"/>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D19" s="2">
         <v>0</v>
       </c>
-      <c r="E19" s="11">
-        <v>1</v>
-      </c>
-      <c r="F19" s="11">
-        <v>1</v>
-      </c>
-      <c r="G19" s="11">
+      <c r="E19" s="10">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10">
+        <v>1</v>
+      </c>
+      <c r="G19" s="10">
         <v>1</v>
       </c>
       <c r="H19" s="2">
@@ -2417,23 +2386,23 @@
       </c>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8"/>
-      <c r="S19" s="8"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="8"/>
-      <c r="V19" s="8"/>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
-      <c r="Y19" s="8"/>
-      <c r="Z19" s="8"/>
-      <c r="AA19" s="8"/>
-      <c r="AB19" s="9" t="s">
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
+      <c r="Z19" s="7"/>
+      <c r="AA19" s="7"/>
+      <c r="AB19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC19" s="6" t="s">
+      <c r="AC19" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AD19" s="1"/>
@@ -2449,25 +2418,25 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>60</v>
       </c>
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="11">
-        <v>1</v>
-      </c>
-      <c r="F20" s="11">
-        <v>1</v>
-      </c>
-      <c r="G20" s="11">
-        <v>1</v>
-      </c>
-      <c r="H20" s="11">
+      <c r="E20" s="10">
+        <v>1</v>
+      </c>
+      <c r="F20" s="10">
+        <v>1</v>
+      </c>
+      <c r="G20" s="10">
+        <v>1</v>
+      </c>
+      <c r="H20" s="10">
         <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
@@ -2480,23 +2449,23 @@
       </c>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8"/>
-      <c r="S20" s="8"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="8"/>
-      <c r="V20" s="8"/>
-      <c r="W20" s="8"/>
-      <c r="X20" s="8"/>
-      <c r="Y20" s="8"/>
-      <c r="Z20" s="8"/>
-      <c r="AA20" s="8"/>
-      <c r="AB20" s="9" t="s">
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
+      <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
+      <c r="Z20" s="7"/>
+      <c r="AA20" s="7"/>
+      <c r="AB20" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC20" s="6" t="s">
+      <c r="AC20" s="3" t="s">
         <v>61</v>
       </c>
       <c r="AD20" s="1"/>
@@ -2512,13 +2481,13 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2"/>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <v>1</v>
       </c>
       <c r="E21" s="2">
@@ -2533,34 +2502,36 @@
       <c r="H21" s="2">
         <v>0</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="2" t="s">
+      <c r="J21" s="16"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="M21" s="16"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="18"/>
+      <c r="S21" s="19"/>
+      <c r="T21" s="19"/>
+      <c r="U21" s="19"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="19"/>
+      <c r="X21" s="19"/>
+      <c r="Y21" s="19"/>
+      <c r="Z21" s="19"/>
+      <c r="AA21" s="20"/>
+      <c r="AB21" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC21" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
-      <c r="Z21" s="2"/>
-      <c r="AA21" s="2"/>
-      <c r="AB21" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC21" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="AD21" s="1"/>
       <c r="AE21" s="1"/>
@@ -2576,13 +2547,13 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="11">
+      <c r="D22" s="10">
         <v>1</v>
       </c>
       <c r="E22" s="2">
@@ -2594,7 +2565,7 @@
       <c r="G22" s="2">
         <v>0</v>
       </c>
-      <c r="H22" s="11">
+      <c r="H22" s="10">
         <v>1</v>
       </c>
       <c r="I22" s="1" t="s">
@@ -2603,7 +2574,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -2620,10 +2591,10 @@
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
       <c r="AA22" s="2"/>
-      <c r="AB22" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC22" s="6" t="s">
+      <c r="AB22" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC22" s="3" t="s">
         <v>68</v>
       </c>
       <c r="AD22" s="1"/>
@@ -2640,13 +2611,13 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <v>1</v>
       </c>
       <c r="E23" s="2">
@@ -2655,11 +2626,11 @@
       <c r="F23" s="2">
         <v>0</v>
       </c>
-      <c r="G23" s="11">
-        <v>1</v>
-      </c>
-      <c r="H23" s="11">
-        <v>1</v>
+      <c r="G23" s="10">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2">
+        <v>0</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>18</v>
@@ -2667,7 +2638,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -2684,10 +2655,10 @@
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
-      <c r="AB23" s="13" t="s">
+      <c r="AB23" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC23" s="6" t="s">
+      <c r="AC23" s="3" t="s">
         <v>71</v>
       </c>
       <c r="AD23" s="1"/>
@@ -2697,26 +2668,26 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="10">
         <v>1</v>
       </c>
       <c r="E24" s="2">
         <v>0</v>
       </c>
-      <c r="F24" s="11">
-        <v>1</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2">
-        <v>0</v>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="10">
+        <v>1</v>
+      </c>
+      <c r="H24" s="10">
+        <v>1</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>18</v>
@@ -2724,7 +2695,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
@@ -2741,10 +2712,10 @@
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
       <c r="AA24" s="2"/>
-      <c r="AB24" s="13" t="s">
+      <c r="AB24" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC24" s="6" t="s">
+      <c r="AC24" s="3" t="s">
         <v>74</v>
       </c>
       <c r="AD24" s="1"/>
@@ -2754,54 +2725,54 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <v>1</v>
       </c>
       <c r="E25" s="2">
         <v>0</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <v>1</v>
       </c>
       <c r="G25" s="2">
         <v>0</v>
       </c>
-      <c r="H25" s="11">
-        <v>1</v>
-      </c>
-      <c r="I25" s="17" t="s">
+      <c r="H25" s="2">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="M25" s="18"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="18"/>
-      <c r="Q25" s="18"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="18"/>
-      <c r="T25" s="18"/>
-      <c r="U25" s="18"/>
-      <c r="V25" s="18"/>
-      <c r="W25" s="18"/>
-      <c r="X25" s="18"/>
-      <c r="Y25" s="18"/>
-      <c r="Z25" s="18"/>
-      <c r="AA25" s="18"/>
-      <c r="AB25" s="13" t="s">
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="2"/>
+      <c r="W25" s="2"/>
+      <c r="X25" s="2"/>
+      <c r="Y25" s="2"/>
+      <c r="Z25" s="2"/>
+      <c r="AA25" s="2"/>
+      <c r="AB25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC25" s="19" t="s">
+      <c r="AC25" s="3" t="s">
         <v>77</v>
       </c>
       <c r="AD25" s="1"/>
@@ -2811,53 +2782,55 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2"/>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="10">
         <v>1</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
       </c>
-      <c r="F26" s="11">
-        <v>1</v>
-      </c>
-      <c r="G26" s="11">
-        <v>1</v>
-      </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="18" t="s">
+      <c r="F26" s="10">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="10">
+        <v>1</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22"/>
+      <c r="Q26" s="22"/>
+      <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="22"/>
+      <c r="U26" s="22"/>
+      <c r="V26" s="22"/>
+      <c r="W26" s="22"/>
+      <c r="X26" s="22"/>
+      <c r="Y26" s="22"/>
+      <c r="Z26" s="22"/>
+      <c r="AA26" s="22"/>
+      <c r="AB26" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC26" s="23" t="s">
         <v>80</v>
-      </c>
-      <c r="L26" s="18"/>
-      <c r="M26" s="18"/>
-      <c r="N26" s="18"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="18"/>
-      <c r="Q26" s="18"/>
-      <c r="R26" s="18"/>
-      <c r="S26" s="18"/>
-      <c r="T26" s="18"/>
-      <c r="U26" s="18"/>
-      <c r="V26" s="18"/>
-      <c r="W26" s="21"/>
-      <c r="X26" s="21"/>
-      <c r="Y26" s="21"/>
-      <c r="Z26" s="21"/>
-      <c r="AA26" s="21"/>
-      <c r="AB26" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC26" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="AD26" s="1"/>
       <c r="AE26" s="1"/>
@@ -2866,55 +2839,53 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2"/>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="D27" s="10">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0</v>
+      </c>
+      <c r="F27" s="10">
+        <v>1</v>
+      </c>
+      <c r="G27" s="10">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="11">
-        <v>1</v>
-      </c>
-      <c r="E27" s="2">
-        <v>0</v>
-      </c>
-      <c r="F27" s="11">
-        <v>1</v>
-      </c>
-      <c r="G27" s="11">
-        <v>1</v>
-      </c>
-      <c r="H27" s="11">
-        <v>1</v>
-      </c>
-      <c r="I27" s="17" t="s">
+      <c r="L27" s="22"/>
+      <c r="M27" s="22"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="22"/>
+      <c r="Q27" s="22"/>
+      <c r="R27" s="22"/>
+      <c r="S27" s="22"/>
+      <c r="T27" s="22"/>
+      <c r="U27" s="22"/>
+      <c r="V27" s="22"/>
+      <c r="W27" s="25"/>
+      <c r="X27" s="25"/>
+      <c r="Y27" s="25"/>
+      <c r="Z27" s="25"/>
+      <c r="AA27" s="25"/>
+      <c r="AB27" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC27" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="J27" s="17"/>
-      <c r="K27" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="L27" s="18"/>
-      <c r="M27" s="18"/>
-      <c r="N27" s="18"/>
-      <c r="O27" s="18"/>
-      <c r="P27" s="18"/>
-      <c r="Q27" s="18"/>
-      <c r="R27" s="18"/>
-      <c r="S27" s="18"/>
-      <c r="T27" s="18"/>
-      <c r="U27" s="18"/>
-      <c r="V27" s="18"/>
-      <c r="W27" s="21"/>
-      <c r="X27" s="21"/>
-      <c r="Y27" s="21"/>
-      <c r="Z27" s="21"/>
-      <c r="AA27" s="21"/>
-      <c r="AB27" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC27" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="AD27" s="1"/>
       <c r="AE27" s="1"/>
@@ -2923,52 +2894,54 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2"/>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="D28" s="10">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0</v>
+      </c>
+      <c r="F28" s="10">
+        <v>1</v>
+      </c>
+      <c r="G28" s="10">
+        <v>1</v>
+      </c>
+      <c r="H28" s="10">
+        <v>1</v>
+      </c>
+      <c r="I28" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D28" s="11">
-        <v>1</v>
-      </c>
-      <c r="E28" s="11">
-        <v>1</v>
-      </c>
-      <c r="F28" s="2">
-        <v>0</v>
-      </c>
-      <c r="G28" s="2">
-        <v>0</v>
-      </c>
-      <c r="H28" s="2">
-        <v>0</v>
-      </c>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="18"/>
-      <c r="R28" s="18"/>
-      <c r="S28" s="18"/>
-      <c r="T28" s="18"/>
-      <c r="U28" s="18"/>
-      <c r="V28" s="18"/>
-      <c r="W28" s="21"/>
-      <c r="X28" s="21"/>
-      <c r="Y28" s="21"/>
-      <c r="Z28" s="21"/>
-      <c r="AA28" s="21"/>
-      <c r="AB28" s="9" t="s">
+      <c r="J28" s="9"/>
+      <c r="K28" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="22"/>
+      <c r="O28" s="22"/>
+      <c r="P28" s="22"/>
+      <c r="Q28" s="22"/>
+      <c r="R28" s="22"/>
+      <c r="S28" s="22"/>
+      <c r="T28" s="22"/>
+      <c r="U28" s="22"/>
+      <c r="V28" s="22"/>
+      <c r="W28" s="25"/>
+      <c r="X28" s="25"/>
+      <c r="Y28" s="25"/>
+      <c r="Z28" s="25"/>
+      <c r="AA28" s="25"/>
+      <c r="AB28" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC28" s="6" t="s">
+      <c r="AC28" s="3" t="s">
         <v>88</v>
       </c>
       <c r="AD28" s="1"/>
@@ -2985,16 +2958,16 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="2"/>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="11">
-        <v>1</v>
-      </c>
-      <c r="E29" s="11">
+      <c r="D29" s="10">
+        <v>1</v>
+      </c>
+      <c r="E29" s="10">
         <v>1</v>
       </c>
       <c r="F29" s="2">
@@ -3003,12 +2976,14 @@
       <c r="G29" s="2">
         <v>0</v>
       </c>
-      <c r="H29" s="11">
-        <v>1</v>
-      </c>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="22"/>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="22" t="s">
+        <v>83</v>
+      </c>
       <c r="L29" s="22"/>
       <c r="M29" s="22"/>
       <c r="N29" s="22"/>
@@ -3020,15 +2995,15 @@
       <c r="T29" s="22"/>
       <c r="U29" s="22"/>
       <c r="V29" s="22"/>
-      <c r="W29" s="22"/>
-      <c r="X29" s="22"/>
-      <c r="Y29" s="22"/>
-      <c r="Z29" s="22"/>
-      <c r="AA29" s="22"/>
-      <c r="AB29" s="9" t="s">
+      <c r="W29" s="25"/>
+      <c r="X29" s="25"/>
+      <c r="Y29" s="25"/>
+      <c r="Z29" s="25"/>
+      <c r="AA29" s="25"/>
+      <c r="AB29" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC29" s="6" t="s">
+      <c r="AC29" s="3" t="s">
         <v>91</v>
       </c>
       <c r="AD29" s="1"/>
@@ -3045,57 +3020,51 @@
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2"/>
-      <c r="B30" s="23" t="s">
+      <c r="B30" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="C30" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="D30" s="11">
-        <v>1</v>
-      </c>
-      <c r="E30" s="11">
+      <c r="D30" s="10">
+        <v>1</v>
+      </c>
+      <c r="E30" s="10">
         <v>1</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
       </c>
-      <c r="G30" s="11">
-        <v>1</v>
-      </c>
-      <c r="H30" s="2">
-        <v>0</v>
-      </c>
-      <c r="I30" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="M30" s="17"/>
-      <c r="N30" s="17"/>
-      <c r="O30" s="18" t="s">
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="10">
+        <v>1</v>
+      </c>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="26"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="26"/>
+      <c r="U30" s="26"/>
+      <c r="V30" s="26"/>
+      <c r="W30" s="26"/>
+      <c r="X30" s="26"/>
+      <c r="Y30" s="26"/>
+      <c r="Z30" s="26"/>
+      <c r="AA30" s="26"/>
+      <c r="AB30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC30" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="P30" s="18"/>
-      <c r="Q30" s="18"/>
-      <c r="R30" s="18"/>
-      <c r="S30" s="18"/>
-      <c r="T30" s="18"/>
-      <c r="U30" s="18"/>
-      <c r="V30" s="18"/>
-      <c r="W30" s="24"/>
-      <c r="X30" s="24"/>
-      <c r="Y30" s="24"/>
-      <c r="Z30" s="24"/>
-      <c r="AA30" s="24"/>
-      <c r="AB30" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC30" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="AD30" s="1"/>
       <c r="AE30" s="1"/>
@@ -3109,56 +3078,56 @@
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2"/>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="D31" s="10">
+        <v>1</v>
+      </c>
+      <c r="E31" s="10">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0</v>
+      </c>
+      <c r="G31" s="10">
+        <v>1</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9"/>
+      <c r="O31" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="11">
-        <v>1</v>
-      </c>
-      <c r="E31" s="11">
-        <v>1</v>
-      </c>
-      <c r="F31" s="2">
-        <v>0</v>
-      </c>
-      <c r="G31" s="11">
-        <v>1</v>
-      </c>
-      <c r="H31" s="11">
-        <v>1</v>
-      </c>
-      <c r="I31" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="P31" s="18"/>
-      <c r="Q31" s="18"/>
-      <c r="R31" s="18"/>
-      <c r="S31" s="18"/>
-      <c r="T31" s="18"/>
-      <c r="U31" s="18"/>
-      <c r="V31" s="18"/>
-      <c r="W31" s="24"/>
-      <c r="X31" s="24"/>
-      <c r="Y31" s="24"/>
-      <c r="Z31" s="24"/>
-      <c r="AA31" s="24"/>
-      <c r="AB31" s="9" t="s">
+      <c r="P31" s="22"/>
+      <c r="Q31" s="22"/>
+      <c r="R31" s="22"/>
+      <c r="S31" s="22"/>
+      <c r="T31" s="22"/>
+      <c r="U31" s="22"/>
+      <c r="V31" s="22"/>
+      <c r="W31" s="7"/>
+      <c r="X31" s="7"/>
+      <c r="Y31" s="7"/>
+      <c r="Z31" s="7"/>
+      <c r="AA31" s="7"/>
+      <c r="AB31" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC31" s="6" t="s">
+      <c r="AC31" s="3" t="s">
         <v>98</v>
       </c>
       <c r="AD31" s="1"/>
@@ -3173,61 +3142,57 @@
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2"/>
-      <c r="B32" s="25" t="s">
+      <c r="B32" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="C32" s="25" t="s">
+      <c r="C32" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="D32" s="11">
-        <v>1</v>
-      </c>
-      <c r="E32" s="11">
-        <v>1</v>
-      </c>
-      <c r="F32" s="11">
-        <v>1</v>
-      </c>
-      <c r="G32" s="2">
-        <v>0</v>
-      </c>
-      <c r="H32" s="2">
-        <v>0</v>
-      </c>
-      <c r="I32" s="18" t="s">
+      <c r="D32" s="10">
+        <v>1</v>
+      </c>
+      <c r="E32" s="10">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0</v>
+      </c>
+      <c r="G32" s="10">
+        <v>1</v>
+      </c>
+      <c r="H32" s="10">
+        <v>1</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9"/>
+      <c r="O32" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="P32" s="22"/>
+      <c r="Q32" s="22"/>
+      <c r="R32" s="22"/>
+      <c r="S32" s="22"/>
+      <c r="T32" s="22"/>
+      <c r="U32" s="22"/>
+      <c r="V32" s="22"/>
+      <c r="W32" s="7"/>
+      <c r="X32" s="7"/>
+      <c r="Y32" s="7"/>
+      <c r="Z32" s="7"/>
+      <c r="AA32" s="7"/>
+      <c r="AB32" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC32" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="P32" s="17"/>
-      <c r="Q32" s="17"/>
-      <c r="R32" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="S32" s="27"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="V32" s="27"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="29"/>
-      <c r="Y32" s="30"/>
-      <c r="Z32" s="30"/>
-      <c r="AA32" s="31"/>
-      <c r="AB32" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC32" s="32" t="s">
-        <v>105</v>
       </c>
       <c r="AD32" s="1"/>
       <c r="AE32" s="1"/>
@@ -3241,50 +3206,60 @@
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="2"/>
-      <c r="B33" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="D33" s="11">
-        <v>1</v>
-      </c>
-      <c r="E33" s="11">
-        <v>1</v>
-      </c>
-      <c r="F33" s="11">
+      <c r="B33" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="D33" s="10">
+        <v>1</v>
+      </c>
+      <c r="E33" s="10">
+        <v>1</v>
+      </c>
+      <c r="F33" s="10">
         <v>1</v>
       </c>
       <c r="G33" s="2">
         <v>0</v>
       </c>
-      <c r="H33" s="11">
-        <v>1</v>
-      </c>
-      <c r="I33" s="22"/>
+      <c r="H33" s="2">
+        <v>0</v>
+      </c>
+      <c r="I33" s="22" t="s">
+        <v>104</v>
+      </c>
       <c r="J33" s="22"/>
       <c r="K33" s="22"/>
-      <c r="L33" s="22"/>
-      <c r="M33" s="22"/>
-      <c r="N33" s="22"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="22"/>
-      <c r="Q33" s="22"/>
-      <c r="R33" s="22"/>
-      <c r="S33" s="22"/>
-      <c r="T33" s="22"/>
-      <c r="U33" s="22"/>
-      <c r="V33" s="22"/>
-      <c r="W33" s="22"/>
-      <c r="X33" s="22"/>
-      <c r="Y33" s="22"/>
-      <c r="Z33" s="22"/>
-      <c r="AA33" s="22"/>
-      <c r="AB33" s="9" t="s">
+      <c r="L33" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="S33" s="30"/>
+      <c r="T33" s="31"/>
+      <c r="U33" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="V33" s="30"/>
+      <c r="W33" s="31"/>
+      <c r="X33" s="32"/>
+      <c r="Y33" s="33"/>
+      <c r="Z33" s="33"/>
+      <c r="AA33" s="34"/>
+      <c r="AB33" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC33" s="32" t="s">
+      <c r="AC33" s="1" t="s">
         <v>108</v>
       </c>
       <c r="AD33" s="1"/>
@@ -3299,52 +3274,50 @@
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2"/>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="25" t="s">
+      <c r="C34" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="D34" s="11">
-        <v>1</v>
-      </c>
-      <c r="E34" s="11">
-        <v>1</v>
-      </c>
-      <c r="F34" s="11">
-        <v>1</v>
-      </c>
-      <c r="G34" s="11">
-        <v>1</v>
-      </c>
-      <c r="H34" s="2">
-        <v>0</v>
-      </c>
-      <c r="I34" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="21"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="21"/>
-      <c r="O34" s="21"/>
-      <c r="P34" s="21"/>
-      <c r="Q34" s="21"/>
-      <c r="R34" s="21"/>
-      <c r="S34" s="21"/>
-      <c r="T34" s="21"/>
-      <c r="U34" s="21"/>
-      <c r="V34" s="21"/>
-      <c r="W34" s="21"/>
-      <c r="X34" s="21"/>
-      <c r="Y34" s="21"/>
-      <c r="Z34" s="21"/>
-      <c r="AA34" s="21"/>
-      <c r="AB34" s="9" t="s">
+      <c r="D34" s="10">
+        <v>1</v>
+      </c>
+      <c r="E34" s="10">
+        <v>1</v>
+      </c>
+      <c r="F34" s="10">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2">
+        <v>0</v>
+      </c>
+      <c r="H34" s="10">
+        <v>1</v>
+      </c>
+      <c r="I34" s="26"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="26"/>
+      <c r="N34" s="26"/>
+      <c r="O34" s="26"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="26"/>
+      <c r="R34" s="26"/>
+      <c r="S34" s="26"/>
+      <c r="T34" s="26"/>
+      <c r="U34" s="26"/>
+      <c r="V34" s="26"/>
+      <c r="W34" s="26"/>
+      <c r="X34" s="26"/>
+      <c r="Y34" s="26"/>
+      <c r="Z34" s="26"/>
+      <c r="AA34" s="26"/>
+      <c r="AB34" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC34" s="32" t="s">
+      <c r="AC34" s="1" t="s">
         <v>111</v>
       </c>
       <c r="AD34" s="1"/>
@@ -3359,52 +3332,52 @@
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="C35" s="25" t="s">
+      <c r="C35" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="D35" s="11">
-        <v>1</v>
-      </c>
-      <c r="E35" s="11">
-        <v>1</v>
-      </c>
-      <c r="F35" s="11">
-        <v>1</v>
-      </c>
-      <c r="G35" s="11">
-        <v>1</v>
-      </c>
-      <c r="H35" s="11">
-        <v>1</v>
-      </c>
-      <c r="I35" s="17" t="s">
+      <c r="D35" s="10">
+        <v>1</v>
+      </c>
+      <c r="E35" s="10">
+        <v>1</v>
+      </c>
+      <c r="F35" s="10">
+        <v>1</v>
+      </c>
+      <c r="G35" s="10">
+        <v>1</v>
+      </c>
+      <c r="H35" s="2">
+        <v>0</v>
+      </c>
+      <c r="I35" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="21"/>
-      <c r="O35" s="21"/>
-      <c r="P35" s="21"/>
-      <c r="Q35" s="21"/>
-      <c r="R35" s="21"/>
-      <c r="S35" s="21"/>
-      <c r="T35" s="21"/>
-      <c r="U35" s="21"/>
-      <c r="V35" s="21"/>
-      <c r="W35" s="21"/>
-      <c r="X35" s="21"/>
-      <c r="Y35" s="21"/>
-      <c r="Z35" s="21"/>
-      <c r="AA35" s="21"/>
-      <c r="AB35" s="9" t="s">
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+      <c r="Q35" s="25"/>
+      <c r="R35" s="25"/>
+      <c r="S35" s="25"/>
+      <c r="T35" s="25"/>
+      <c r="U35" s="25"/>
+      <c r="V35" s="25"/>
+      <c r="W35" s="25"/>
+      <c r="X35" s="25"/>
+      <c r="Y35" s="25"/>
+      <c r="Z35" s="25"/>
+      <c r="AA35" s="25"/>
+      <c r="AB35" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="AC35" s="32" t="s">
+      <c r="AC35" s="1" t="s">
         <v>114</v>
       </c>
       <c r="AD35" s="1"/>
@@ -3419,34 +3392,54 @@
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="2"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
-      <c r="Q36" s="1"/>
-      <c r="R36" s="1"/>
-      <c r="S36" s="1"/>
-      <c r="T36" s="1"/>
-      <c r="U36" s="1"/>
-      <c r="V36" s="1"/>
-      <c r="W36" s="1"/>
-      <c r="X36" s="1"/>
-      <c r="Y36" s="1"/>
-      <c r="Z36" s="1"/>
-      <c r="AA36" s="1"/>
-      <c r="AB36" s="1"/>
-      <c r="AC36" s="1"/>
+      <c r="B36" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="D36" s="10">
+        <v>1</v>
+      </c>
+      <c r="E36" s="10">
+        <v>1</v>
+      </c>
+      <c r="F36" s="10">
+        <v>1</v>
+      </c>
+      <c r="G36" s="10">
+        <v>1</v>
+      </c>
+      <c r="H36" s="10">
+        <v>1</v>
+      </c>
+      <c r="I36" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="25"/>
+      <c r="M36" s="25"/>
+      <c r="N36" s="25"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="25"/>
+      <c r="Q36" s="25"/>
+      <c r="R36" s="25"/>
+      <c r="S36" s="25"/>
+      <c r="T36" s="25"/>
+      <c r="U36" s="25"/>
+      <c r="V36" s="25"/>
+      <c r="W36" s="25"/>
+      <c r="X36" s="25"/>
+      <c r="Y36" s="25"/>
+      <c r="Z36" s="25"/>
+      <c r="AA36" s="25"/>
+      <c r="AB36" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC36" s="1" t="s">
+        <v>117</v>
+      </c>
       <c r="AD36" s="1"/>
       <c r="AE36" s="1"/>
       <c r="AF36" s="1"/>
@@ -3459,26 +3452,7 @@
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="2"/>
-      <c r="B37" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="34"/>
-      <c r="J37" s="34"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
-      <c r="M37" s="34"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
-      <c r="P37" s="34"/>
-      <c r="Q37" s="34"/>
-      <c r="R37" s="35"/>
-      <c r="S37" s="36"/>
+      <c r="S37" s="4"/>
       <c r="T37" s="1"/>
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
@@ -3501,31 +3475,6 @@
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="2"/>
-      <c r="B38" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
-      <c r="N38" s="3"/>
-      <c r="O38" s="3"/>
-      <c r="P38" s="3"/>
-      <c r="Q38" s="3"/>
-      <c r="R38" s="3"/>
       <c r="T38" s="1"/>
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
@@ -3548,31 +3497,6 @@
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="2"/>
-      <c r="B39" s="37" t="s">
-        <v>118</v>
-      </c>
-      <c r="C39" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
-      <c r="O39" s="3"/>
-      <c r="P39" s="3"/>
-      <c r="Q39" s="3"/>
-      <c r="R39" s="3"/>
       <c r="T39" s="1"/>
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
@@ -3595,31 +3519,6 @@
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="2"/>
-      <c r="B40" s="37" t="s">
-        <v>122</v>
-      </c>
-      <c r="C40" s="37" t="s">
-        <v>123</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="4"/>
-      <c r="K40" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
-      <c r="N40" s="3"/>
-      <c r="O40" s="3"/>
-      <c r="P40" s="3"/>
-      <c r="Q40" s="3"/>
-      <c r="R40" s="3"/>
       <c r="T40" s="1"/>
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
@@ -3642,31 +3541,6 @@
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="2"/>
-      <c r="B41" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="C41" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L41" s="4"/>
-      <c r="M41" s="4"/>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
-      <c r="P41" s="4"/>
-      <c r="Q41" s="4"/>
-      <c r="R41" s="4"/>
       <c r="T41" s="1"/>
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
@@ -3689,31 +3563,6 @@
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="2"/>
-      <c r="B42" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="C42" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="L42" s="4"/>
-      <c r="M42" s="4"/>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
-      <c r="P42" s="4"/>
-      <c r="Q42" s="4"/>
-      <c r="R42" s="4"/>
       <c r="T42" s="1"/>
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
@@ -3735,31 +3584,6 @@
       <c r="AL42" s="1"/>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="B43" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="C43" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="L43" s="4"/>
-      <c r="M43" s="4"/>
-      <c r="N43" s="4"/>
-      <c r="O43" s="4"/>
-      <c r="P43" s="4"/>
-      <c r="Q43" s="4"/>
-      <c r="R43" s="4"/>
       <c r="T43" s="1"/>
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
@@ -3871,15 +3695,25 @@
       <c r="AL46" s="1"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
-      <c r="K47" s="1"/>
-      <c r="L47" s="1"/>
+      <c r="B47" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="36"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="36"/>
+      <c r="H47" s="36"/>
+      <c r="I47" s="36"/>
+      <c r="J47" s="36"/>
+      <c r="K47" s="36"/>
+      <c r="L47" s="36"/>
+      <c r="M47" s="36"/>
+      <c r="N47" s="36"/>
+      <c r="O47" s="36"/>
+      <c r="P47" s="36"/>
+      <c r="Q47" s="36"/>
+      <c r="R47" s="37"/>
       <c r="T47" s="1"/>
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
@@ -3901,15 +3735,31 @@
       <c r="AL47" s="1"/>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
+      <c r="B48" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+      <c r="P48" s="3"/>
+      <c r="Q48" s="3"/>
+      <c r="R48" s="3"/>
       <c r="T48" s="1"/>
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
@@ -3931,15 +3781,31 @@
       <c r="AL48" s="1"/>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="1"/>
+      <c r="B49" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+      <c r="P49" s="3"/>
+      <c r="Q49" s="3"/>
+      <c r="R49" s="3"/>
       <c r="T49" s="1"/>
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
@@ -3961,23 +3827,31 @@
       <c r="AL49" s="1"/>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="1"/>
-      <c r="M50" s="1"/>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-      <c r="P50" s="1"/>
-      <c r="Q50" s="1"/>
-      <c r="R50" s="1"/>
+      <c r="B50" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+      <c r="P50" s="3"/>
+      <c r="Q50" s="3"/>
+      <c r="R50" s="3"/>
       <c r="S50" s="1"/>
       <c r="T50" s="1"/>
       <c r="U50" s="1"/>
@@ -4000,23 +3874,31 @@
       <c r="AL50" s="1"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1"/>
-      <c r="K51" s="1"/>
-      <c r="L51" s="1"/>
-      <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-      <c r="O51" s="1"/>
-      <c r="P51" s="1"/>
-      <c r="Q51" s="1"/>
-      <c r="R51" s="1"/>
+      <c r="B51" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="C51" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="4"/>
       <c r="S51" s="1"/>
       <c r="T51" s="1"/>
       <c r="U51" s="1"/>
@@ -4039,23 +3921,31 @@
       <c r="AL51" s="1"/>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="1"/>
-      <c r="J52" s="1"/>
-      <c r="K52" s="1"/>
-      <c r="L52" s="1"/>
-      <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-      <c r="P52" s="1"/>
-      <c r="Q52" s="1"/>
-      <c r="R52" s="1"/>
+      <c r="B52" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="C52" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="4"/>
       <c r="S52" s="1"/>
       <c r="T52" s="1"/>
       <c r="U52" s="1"/>
@@ -4078,23 +3968,31 @@
       <c r="AL52" s="1"/>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="1"/>
-      <c r="J53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-      <c r="P53" s="1"/>
-      <c r="Q53" s="1"/>
-      <c r="R53" s="1"/>
+      <c r="B53" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="4"/>
       <c r="S53" s="1"/>
       <c r="T53" s="1"/>
       <c r="U53" s="1"/>
@@ -4627,10 +4525,10 @@
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="38"/>
-      <c r="F67" s="38"/>
-      <c r="G67" s="38"/>
-      <c r="H67" s="38"/>
+      <c r="E67" s="39"/>
+      <c r="F67" s="39"/>
+      <c r="G67" s="39"/>
+      <c r="H67" s="39"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
@@ -4666,10 +4564,10 @@
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="38"/>
-      <c r="F68" s="38"/>
-      <c r="G68" s="38"/>
-      <c r="H68" s="38"/>
+      <c r="E68" s="39"/>
+      <c r="F68" s="39"/>
+      <c r="G68" s="39"/>
+      <c r="H68" s="39"/>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
@@ -4705,10 +4603,10 @@
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
-      <c r="E69" s="38"/>
-      <c r="F69" s="38"/>
-      <c r="G69" s="38"/>
-      <c r="H69" s="38"/>
+      <c r="E69" s="39"/>
+      <c r="F69" s="39"/>
+      <c r="G69" s="39"/>
+      <c r="H69" s="39"/>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
@@ -4744,10 +4642,10 @@
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
-      <c r="E70" s="38"/>
-      <c r="F70" s="38"/>
-      <c r="G70" s="38"/>
-      <c r="H70" s="38"/>
+      <c r="E70" s="39"/>
+      <c r="F70" s="39"/>
+      <c r="G70" s="39"/>
+      <c r="H70" s="39"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
@@ -4783,10 +4681,10 @@
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="38"/>
-      <c r="F71" s="38"/>
-      <c r="G71" s="38"/>
-      <c r="H71" s="38"/>
+      <c r="E71" s="39"/>
+      <c r="F71" s="39"/>
+      <c r="G71" s="39"/>
+      <c r="H71" s="39"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -4822,10 +4720,10 @@
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="38"/>
-      <c r="F72" s="38"/>
-      <c r="G72" s="38"/>
-      <c r="H72" s="38"/>
+      <c r="E72" s="39"/>
+      <c r="F72" s="39"/>
+      <c r="G72" s="39"/>
+      <c r="H72" s="39"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
@@ -4866,7 +4764,7 @@
     <row r="79" ht="15" customHeight="1"/>
     <row r="80" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="112">
+  <mergeCells count="116">
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="L2:S2"/>
     <mergeCell ref="T2:AA2"/>
@@ -4928,7 +4826,9 @@
     <mergeCell ref="L20:N20"/>
     <mergeCell ref="O20:AA20"/>
     <mergeCell ref="I21:K21"/>
-    <mergeCell ref="L21:AA21"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="R21:AA21"/>
     <mergeCell ref="I22:K22"/>
     <mergeCell ref="L22:AA22"/>
     <mergeCell ref="I23:K23"/>
@@ -4937,48 +4837,50 @@
     <mergeCell ref="L24:AA24"/>
     <mergeCell ref="I25:K25"/>
     <mergeCell ref="L25:AA25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="K26:V26"/>
-    <mergeCell ref="W26:AA26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L26:AA26"/>
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="K27:V27"/>
     <mergeCell ref="W27:AA27"/>
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="K28:V28"/>
     <mergeCell ref="W28:AA28"/>
-    <mergeCell ref="I29:AA29"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="O30:V30"/>
-    <mergeCell ref="W30:AA30"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="K29:V29"/>
+    <mergeCell ref="W29:AA29"/>
+    <mergeCell ref="I30:AA30"/>
     <mergeCell ref="I31:K31"/>
     <mergeCell ref="L31:N31"/>
     <mergeCell ref="O31:V31"/>
     <mergeCell ref="W31:AA31"/>
     <mergeCell ref="I32:K32"/>
     <mergeCell ref="L32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="R32:T32"/>
-    <mergeCell ref="U32:W32"/>
-    <mergeCell ref="X32:AA32"/>
-    <mergeCell ref="I33:AA33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="L34:AA34"/>
+    <mergeCell ref="O32:V32"/>
+    <mergeCell ref="W32:AA32"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="R33:T33"/>
+    <mergeCell ref="U33:W33"/>
+    <mergeCell ref="X33:AA33"/>
+    <mergeCell ref="I34:AA34"/>
     <mergeCell ref="I35:K35"/>
     <mergeCell ref="L35:AA35"/>
-    <mergeCell ref="B37:R37"/>
-    <mergeCell ref="D38:J38"/>
-    <mergeCell ref="K38:R38"/>
-    <mergeCell ref="D39:J39"/>
-    <mergeCell ref="K39:R39"/>
-    <mergeCell ref="D40:J40"/>
-    <mergeCell ref="K40:R40"/>
-    <mergeCell ref="D41:J41"/>
-    <mergeCell ref="K41:R41"/>
-    <mergeCell ref="D42:J42"/>
-    <mergeCell ref="K42:R42"/>
-    <mergeCell ref="D43:J43"/>
-    <mergeCell ref="K43:R43"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="L36:AA36"/>
+    <mergeCell ref="B47:R47"/>
+    <mergeCell ref="D48:J48"/>
+    <mergeCell ref="K48:R48"/>
+    <mergeCell ref="D49:J49"/>
+    <mergeCell ref="K49:R49"/>
+    <mergeCell ref="D50:J50"/>
+    <mergeCell ref="K50:R50"/>
+    <mergeCell ref="D51:J51"/>
+    <mergeCell ref="K51:R51"/>
+    <mergeCell ref="D52:J52"/>
+    <mergeCell ref="K52:R52"/>
+    <mergeCell ref="D53:J53"/>
+    <mergeCell ref="K53:R53"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Extend demo, change SHF to ROL, a circular shift
</commit_message>
<xml_diff>
--- a/Xis16 Spreadsheet.xlsx
+++ b/Xis16 Spreadsheet.xlsx
@@ -204,13 +204,13 @@
     <t xml:space="preserve">C &lt;- A &lt;&lt; 1 (physical shift)</t>
   </si>
   <si>
-    <t>SHF</t>
-  </si>
-  <si>
-    <t>Shift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C &lt;- A &gt;&gt; B </t>
+    <t>ROL</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C &lt;- (A &gt;&gt; B) | (A &lt;&lt; (n - B))</t>
   </si>
   <si>
     <t>LDI</t>

</xml_diff>

<commit_message>
Implement a syntax checker that throws an error if the syntax is wrong
</commit_message>
<xml_diff>
--- a/Xis16 Spreadsheet.xlsx
+++ b/Xis16 Spreadsheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t xml:space="preserve">Byte 1</t>
   </si>
@@ -336,10 +336,7 @@
     <t xml:space="preserve">Reg Y</t>
   </si>
   <si>
-    <t xml:space="preserve">Reg R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg G</t>
+    <t xml:space="preserve">Reg RGB</t>
   </si>
   <si>
     <t xml:space="preserve">Buffer &lt;- X || Y || RGB</t>
@@ -560,7 +557,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -620,11 +617,48 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="37">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -710,22 +744,13 @@
     <xf fontId="1" fillId="15" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3242,25 +3267,21 @@
       </c>
       <c r="P33" s="9"/>
       <c r="Q33" s="9"/>
-      <c r="R33" s="29" t="s">
-        <v>107</v>
-      </c>
+      <c r="R33" s="29"/>
       <c r="S33" s="30"/>
-      <c r="T33" s="31"/>
-      <c r="U33" s="29" t="s">
-        <v>19</v>
-      </c>
+      <c r="T33" s="30"/>
+      <c r="U33" s="30"/>
       <c r="V33" s="30"/>
-      <c r="W33" s="31"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="33"/>
-      <c r="Z33" s="33"/>
-      <c r="AA33" s="34"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="30"/>
+      <c r="Y33" s="30"/>
+      <c r="Z33" s="30"/>
+      <c r="AA33" s="31"/>
       <c r="AB33" s="8" t="s">
         <v>11</v>
       </c>
       <c r="AC33" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD33" s="1"/>
       <c r="AE33" s="1"/>
@@ -3275,10 +3296,10 @@
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2"/>
       <c r="B34" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" s="28" t="s">
         <v>109</v>
-      </c>
-      <c r="C34" s="28" t="s">
-        <v>110</v>
       </c>
       <c r="D34" s="10">
         <v>1</v>
@@ -3318,7 +3339,7 @@
         <v>11</v>
       </c>
       <c r="AC34" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AD34" s="1"/>
       <c r="AE34" s="1"/>
@@ -3333,10 +3354,10 @@
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="2"/>
       <c r="B35" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" s="28" t="s">
         <v>112</v>
-      </c>
-      <c r="C35" s="28" t="s">
-        <v>113</v>
       </c>
       <c r="D35" s="10">
         <v>1</v>
@@ -3378,7 +3399,7 @@
         <v>11</v>
       </c>
       <c r="AC35" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AD35" s="1"/>
       <c r="AE35" s="1"/>
@@ -3393,10 +3414,10 @@
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="2"/>
       <c r="B36" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36" s="28" t="s">
         <v>115</v>
-      </c>
-      <c r="C36" s="28" t="s">
-        <v>116</v>
       </c>
       <c r="D36" s="10">
         <v>1</v>
@@ -3438,7 +3459,7 @@
         <v>11</v>
       </c>
       <c r="AC36" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AD36" s="1"/>
       <c r="AE36" s="1"/>
@@ -3695,25 +3716,25 @@
       <c r="AL46" s="1"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="B47" s="35" t="s">
-        <v>118</v>
-      </c>
-      <c r="C47" s="36"/>
-      <c r="D47" s="36"/>
-      <c r="E47" s="36"/>
-      <c r="F47" s="36"/>
-      <c r="G47" s="36"/>
-      <c r="H47" s="36"/>
-      <c r="I47" s="36"/>
-      <c r="J47" s="36"/>
-      <c r="K47" s="36"/>
-      <c r="L47" s="36"/>
-      <c r="M47" s="36"/>
-      <c r="N47" s="36"/>
-      <c r="O47" s="36"/>
-      <c r="P47" s="36"/>
-      <c r="Q47" s="36"/>
-      <c r="R47" s="37"/>
+      <c r="B47" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
+      <c r="M47" s="33"/>
+      <c r="N47" s="33"/>
+      <c r="O47" s="33"/>
+      <c r="P47" s="33"/>
+      <c r="Q47" s="33"/>
+      <c r="R47" s="34"/>
       <c r="T47" s="1"/>
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
@@ -3742,7 +3763,7 @@
         <v>4</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -3751,7 +3772,7 @@
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
@@ -3781,14 +3802,14 @@
       <c r="AL48" s="1"/>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="B49" s="38" t="s">
+      <c r="B49" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C49" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="C49" s="38" t="s">
+      <c r="D49" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
@@ -3797,7 +3818,7 @@
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
       <c r="K49" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
@@ -3827,14 +3848,14 @@
       <c r="AL49" s="1"/>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="38" t="s">
+      <c r="B50" s="35" t="s">
+        <v>124</v>
+      </c>
+      <c r="C50" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="C50" s="38" t="s">
+      <c r="D50" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
@@ -3843,7 +3864,7 @@
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
       <c r="K50" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L50" s="3"/>
       <c r="M50" s="3"/>
@@ -3874,14 +3895,14 @@
       <c r="AL50" s="1"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="B51" s="38" t="s">
+      <c r="B51" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="C51" s="38" t="s">
+      <c r="D51" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>131</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
@@ -3890,7 +3911,7 @@
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
       <c r="K51" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L51" s="4"/>
       <c r="M51" s="4"/>
@@ -3921,14 +3942,14 @@
       <c r="AL51" s="1"/>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="B52" s="38" t="s">
+      <c r="B52" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C52" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="C52" s="38" t="s">
+      <c r="D52" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
@@ -3937,7 +3958,7 @@
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
       <c r="K52" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L52" s="4"/>
       <c r="M52" s="4"/>
@@ -3968,14 +3989,14 @@
       <c r="AL52" s="1"/>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="B53" s="38" t="s">
+      <c r="B53" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="C53" s="35" t="s">
         <v>137</v>
       </c>
-      <c r="C53" s="38" t="s">
+      <c r="D53" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
@@ -3984,7 +4005,7 @@
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
       <c r="K53" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L53" s="4"/>
       <c r="M53" s="4"/>
@@ -4525,10 +4546,10 @@
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="39"/>
-      <c r="F67" s="39"/>
-      <c r="G67" s="39"/>
-      <c r="H67" s="39"/>
+      <c r="E67" s="36"/>
+      <c r="F67" s="36"/>
+      <c r="G67" s="36"/>
+      <c r="H67" s="36"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
@@ -4564,10 +4585,10 @@
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="39"/>
-      <c r="F68" s="39"/>
-      <c r="G68" s="39"/>
-      <c r="H68" s="39"/>
+      <c r="E68" s="36"/>
+      <c r="F68" s="36"/>
+      <c r="G68" s="36"/>
+      <c r="H68" s="36"/>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
@@ -4603,10 +4624,10 @@
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
-      <c r="E69" s="39"/>
-      <c r="F69" s="39"/>
-      <c r="G69" s="39"/>
-      <c r="H69" s="39"/>
+      <c r="E69" s="36"/>
+      <c r="F69" s="36"/>
+      <c r="G69" s="36"/>
+      <c r="H69" s="36"/>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
@@ -4642,10 +4663,10 @@
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
-      <c r="E70" s="39"/>
-      <c r="F70" s="39"/>
-      <c r="G70" s="39"/>
-      <c r="H70" s="39"/>
+      <c r="E70" s="36"/>
+      <c r="F70" s="36"/>
+      <c r="G70" s="36"/>
+      <c r="H70" s="36"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
@@ -4681,10 +4702,10 @@
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="39"/>
-      <c r="F71" s="39"/>
-      <c r="G71" s="39"/>
-      <c r="H71" s="39"/>
+      <c r="E71" s="36"/>
+      <c r="F71" s="36"/>
+      <c r="G71" s="36"/>
+      <c r="H71" s="36"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -4720,10 +4741,10 @@
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="39"/>
-      <c r="F72" s="39"/>
-      <c r="G72" s="39"/>
-      <c r="H72" s="39"/>
+      <c r="E72" s="36"/>
+      <c r="F72" s="36"/>
+      <c r="G72" s="36"/>
+      <c r="H72" s="36"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
@@ -4764,7 +4785,7 @@
     <row r="79" ht="15" customHeight="1"/>
     <row r="80" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="116">
+  <mergeCells count="114">
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="L2:S2"/>
     <mergeCell ref="T2:AA2"/>
@@ -4860,9 +4881,7 @@
     <mergeCell ref="I33:K33"/>
     <mergeCell ref="L33:N33"/>
     <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="R33:T33"/>
-    <mergeCell ref="U33:W33"/>
-    <mergeCell ref="X33:AA33"/>
+    <mergeCell ref="R33:AA33"/>
     <mergeCell ref="I34:AA34"/>
     <mergeCell ref="I35:K35"/>
     <mergeCell ref="L35:AA35"/>

</xml_diff>

<commit_message>
Update Xis16 Spreadsheet, fix critical mistake
</commit_message>
<xml_diff>
--- a/Xis16 Spreadsheet.xlsx
+++ b/Xis16 Spreadsheet.xlsx
@@ -557,7 +557,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="11">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -569,43 +569,6 @@
       <left style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </left>
-      <right style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
       <right style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </right>
@@ -654,11 +617,85 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right style="none"/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="46">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -702,6 +739,15 @@
     <xf fontId="1" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="1" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -711,13 +757,31 @@
     <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="5" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -744,22 +808,22 @@
     <xf fontId="1" fillId="15" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="16" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2343,24 +2407,24 @@
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
-      <c r="L18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-      <c r="S18" s="7"/>
-      <c r="T18" s="7"/>
-      <c r="U18" s="7"/>
-      <c r="V18" s="7"/>
-      <c r="W18" s="7"/>
-      <c r="X18" s="7"/>
-      <c r="Y18" s="7"/>
-      <c r="Z18" s="7"/>
-      <c r="AA18" s="7"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="P18" s="19"/>
+      <c r="Q18" s="20"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="22"/>
+      <c r="T18" s="22"/>
+      <c r="U18" s="22"/>
+      <c r="V18" s="22"/>
+      <c r="W18" s="22"/>
+      <c r="X18" s="22"/>
+      <c r="Y18" s="22"/>
+      <c r="Z18" s="22"/>
+      <c r="AA18" s="23"/>
       <c r="AB18" s="12" t="s">
         <v>21</v>
       </c>
@@ -2406,24 +2470,24 @@
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
-      <c r="L19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="7"/>
-      <c r="S19" s="7"/>
-      <c r="T19" s="7"/>
-      <c r="U19" s="7"/>
-      <c r="V19" s="7"/>
-      <c r="W19" s="7"/>
-      <c r="X19" s="7"/>
-      <c r="Y19" s="7"/>
-      <c r="Z19" s="7"/>
-      <c r="AA19" s="7"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="20"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="16"/>
+      <c r="X19" s="16"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="17"/>
       <c r="AB19" s="8" t="s">
         <v>11</v>
       </c>
@@ -2469,24 +2533,24 @@
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-      <c r="L20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="7"/>
-      <c r="V20" s="7"/>
-      <c r="W20" s="7"/>
-      <c r="X20" s="7"/>
-      <c r="Y20" s="7"/>
-      <c r="Z20" s="7"/>
-      <c r="AA20" s="7"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="20"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="22"/>
+      <c r="T20" s="22"/>
+      <c r="U20" s="22"/>
+      <c r="V20" s="22"/>
+      <c r="W20" s="22"/>
+      <c r="X20" s="22"/>
+      <c r="Y20" s="22"/>
+      <c r="Z20" s="22"/>
+      <c r="AA20" s="23"/>
       <c r="AB20" s="8" t="s">
         <v>11</v>
       </c>
@@ -2527,31 +2591,31 @@
       <c r="H21" s="2">
         <v>0</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="16"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="15" t="s">
+      <c r="J21" s="25"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="15" t="s">
+      <c r="M21" s="25"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="P21" s="16"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="18"/>
-      <c r="S21" s="19"/>
-      <c r="T21" s="19"/>
-      <c r="U21" s="19"/>
-      <c r="V21" s="19"/>
-      <c r="W21" s="19"/>
-      <c r="X21" s="19"/>
-      <c r="Y21" s="19"/>
-      <c r="Z21" s="19"/>
-      <c r="AA21" s="20"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="26"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
+      <c r="V21" s="28"/>
+      <c r="W21" s="28"/>
+      <c r="X21" s="28"/>
+      <c r="Y21" s="28"/>
+      <c r="Z21" s="28"/>
+      <c r="AA21" s="29"/>
       <c r="AB21" s="8" t="s">
         <v>11</v>
       </c>
@@ -2572,10 +2636,10 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="30" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="10">
@@ -2636,10 +2700,10 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="30" t="s">
         <v>70</v>
       </c>
       <c r="D23" s="10">
@@ -2693,10 +2757,10 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="30" t="s">
         <v>73</v>
       </c>
       <c r="D24" s="10">
@@ -2750,10 +2814,10 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="30" t="s">
         <v>76</v>
       </c>
       <c r="D25" s="10">
@@ -2807,10 +2871,10 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2"/>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="30" t="s">
         <v>79</v>
       </c>
       <c r="D26" s="10">
@@ -2833,28 +2897,28 @@
       </c>
       <c r="J26" s="9"/>
       <c r="K26" s="9"/>
-      <c r="L26" s="22" t="s">
+      <c r="L26" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="M26" s="22"/>
-      <c r="N26" s="22"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="22"/>
-      <c r="Q26" s="22"/>
-      <c r="R26" s="22"/>
-      <c r="S26" s="22"/>
-      <c r="T26" s="22"/>
-      <c r="U26" s="22"/>
-      <c r="V26" s="22"/>
-      <c r="W26" s="22"/>
-      <c r="X26" s="22"/>
-      <c r="Y26" s="22"/>
-      <c r="Z26" s="22"/>
-      <c r="AA26" s="22"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
+      <c r="O26" s="31"/>
+      <c r="P26" s="31"/>
+      <c r="Q26" s="31"/>
+      <c r="R26" s="31"/>
+      <c r="S26" s="31"/>
+      <c r="T26" s="31"/>
+      <c r="U26" s="31"/>
+      <c r="V26" s="31"/>
+      <c r="W26" s="31"/>
+      <c r="X26" s="31"/>
+      <c r="Y26" s="31"/>
+      <c r="Z26" s="31"/>
+      <c r="AA26" s="31"/>
       <c r="AB26" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AC26" s="23" t="s">
+      <c r="AC26" s="32" t="s">
         <v>80</v>
       </c>
       <c r="AD26" s="1"/>
@@ -2864,10 +2928,10 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2"/>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="33" t="s">
         <v>82</v>
       </c>
       <c r="D27" s="10">
@@ -2885,27 +2949,27 @@
       <c r="H27" s="2">
         <v>0</v>
       </c>
-      <c r="I27" s="25"/>
-      <c r="J27" s="25"/>
-      <c r="K27" s="22" t="s">
+      <c r="I27" s="34"/>
+      <c r="J27" s="34"/>
+      <c r="K27" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
-      <c r="R27" s="22"/>
-      <c r="S27" s="22"/>
-      <c r="T27" s="22"/>
-      <c r="U27" s="22"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="25"/>
-      <c r="X27" s="25"/>
-      <c r="Y27" s="25"/>
-      <c r="Z27" s="25"/>
-      <c r="AA27" s="25"/>
+      <c r="L27" s="31"/>
+      <c r="M27" s="31"/>
+      <c r="N27" s="31"/>
+      <c r="O27" s="31"/>
+      <c r="P27" s="31"/>
+      <c r="Q27" s="31"/>
+      <c r="R27" s="31"/>
+      <c r="S27" s="31"/>
+      <c r="T27" s="31"/>
+      <c r="U27" s="31"/>
+      <c r="V27" s="31"/>
+      <c r="W27" s="34"/>
+      <c r="X27" s="34"/>
+      <c r="Y27" s="34"/>
+      <c r="Z27" s="34"/>
+      <c r="AA27" s="34"/>
       <c r="AB27" s="8" t="s">
         <v>11</v>
       </c>
@@ -2919,10 +2983,10 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2"/>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="33" t="s">
         <v>86</v>
       </c>
       <c r="D28" s="10">
@@ -2944,25 +3008,25 @@
         <v>87</v>
       </c>
       <c r="J28" s="9"/>
-      <c r="K28" s="22" t="s">
+      <c r="K28" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="L28" s="22"/>
-      <c r="M28" s="22"/>
-      <c r="N28" s="22"/>
-      <c r="O28" s="22"/>
-      <c r="P28" s="22"/>
-      <c r="Q28" s="22"/>
-      <c r="R28" s="22"/>
-      <c r="S28" s="22"/>
-      <c r="T28" s="22"/>
-      <c r="U28" s="22"/>
-      <c r="V28" s="22"/>
-      <c r="W28" s="25"/>
-      <c r="X28" s="25"/>
-      <c r="Y28" s="25"/>
-      <c r="Z28" s="25"/>
-      <c r="AA28" s="25"/>
+      <c r="L28" s="31"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
+      <c r="R28" s="31"/>
+      <c r="S28" s="31"/>
+      <c r="T28" s="31"/>
+      <c r="U28" s="31"/>
+      <c r="V28" s="31"/>
+      <c r="W28" s="34"/>
+      <c r="X28" s="34"/>
+      <c r="Y28" s="34"/>
+      <c r="Z28" s="34"/>
+      <c r="AA28" s="34"/>
       <c r="AB28" s="8" t="s">
         <v>11</v>
       </c>
@@ -2983,10 +3047,10 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="2"/>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="33" t="s">
         <v>90</v>
       </c>
       <c r="D29" s="10">
@@ -3004,27 +3068,27 @@
       <c r="H29" s="2">
         <v>0</v>
       </c>
-      <c r="I29" s="25"/>
-      <c r="J29" s="25"/>
-      <c r="K29" s="22" t="s">
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="22"/>
-      <c r="P29" s="22"/>
-      <c r="Q29" s="22"/>
-      <c r="R29" s="22"/>
-      <c r="S29" s="22"/>
-      <c r="T29" s="22"/>
-      <c r="U29" s="22"/>
-      <c r="V29" s="22"/>
-      <c r="W29" s="25"/>
-      <c r="X29" s="25"/>
-      <c r="Y29" s="25"/>
-      <c r="Z29" s="25"/>
-      <c r="AA29" s="25"/>
+      <c r="L29" s="31"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="31"/>
+      <c r="P29" s="31"/>
+      <c r="Q29" s="31"/>
+      <c r="R29" s="31"/>
+      <c r="S29" s="31"/>
+      <c r="T29" s="31"/>
+      <c r="U29" s="31"/>
+      <c r="V29" s="31"/>
+      <c r="W29" s="34"/>
+      <c r="X29" s="34"/>
+      <c r="Y29" s="34"/>
+      <c r="Z29" s="34"/>
+      <c r="AA29" s="34"/>
       <c r="AB29" s="8" t="s">
         <v>11</v>
       </c>
@@ -3045,10 +3109,10 @@
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2"/>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="33" t="s">
         <v>93</v>
       </c>
       <c r="D30" s="10">
@@ -3066,25 +3130,25 @@
       <c r="H30" s="10">
         <v>1</v>
       </c>
-      <c r="I30" s="26"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="26"/>
-      <c r="L30" s="26"/>
-      <c r="M30" s="26"/>
-      <c r="N30" s="26"/>
-      <c r="O30" s="26"/>
-      <c r="P30" s="26"/>
-      <c r="Q30" s="26"/>
-      <c r="R30" s="26"/>
-      <c r="S30" s="26"/>
-      <c r="T30" s="26"/>
-      <c r="U30" s="26"/>
-      <c r="V30" s="26"/>
-      <c r="W30" s="26"/>
-      <c r="X30" s="26"/>
-      <c r="Y30" s="26"/>
-      <c r="Z30" s="26"/>
-      <c r="AA30" s="26"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="35"/>
+      <c r="R30" s="35"/>
+      <c r="S30" s="35"/>
+      <c r="T30" s="35"/>
+      <c r="U30" s="35"/>
+      <c r="V30" s="35"/>
+      <c r="W30" s="35"/>
+      <c r="X30" s="35"/>
+      <c r="Y30" s="35"/>
+      <c r="Z30" s="35"/>
+      <c r="AA30" s="35"/>
       <c r="AB30" s="8" t="s">
         <v>11</v>
       </c>
@@ -3103,10 +3167,10 @@
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2"/>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="27" t="s">
+      <c r="C31" s="36" t="s">
         <v>96</v>
       </c>
       <c r="D31" s="10">
@@ -3134,16 +3198,16 @@
       </c>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="22" t="s">
+      <c r="O31" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="P31" s="22"/>
-      <c r="Q31" s="22"/>
-      <c r="R31" s="22"/>
-      <c r="S31" s="22"/>
-      <c r="T31" s="22"/>
-      <c r="U31" s="22"/>
-      <c r="V31" s="22"/>
+      <c r="P31" s="31"/>
+      <c r="Q31" s="31"/>
+      <c r="R31" s="31"/>
+      <c r="S31" s="31"/>
+      <c r="T31" s="31"/>
+      <c r="U31" s="31"/>
+      <c r="V31" s="31"/>
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
       <c r="Y31" s="7"/>
@@ -3167,10 +3231,10 @@
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2"/>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="C32" s="27" t="s">
+      <c r="C32" s="36" t="s">
         <v>100</v>
       </c>
       <c r="D32" s="10">
@@ -3198,16 +3262,16 @@
       </c>
       <c r="M32" s="9"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="22" t="s">
+      <c r="O32" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="P32" s="22"/>
-      <c r="Q32" s="22"/>
-      <c r="R32" s="22"/>
-      <c r="S32" s="22"/>
-      <c r="T32" s="22"/>
-      <c r="U32" s="22"/>
-      <c r="V32" s="22"/>
+      <c r="P32" s="31"/>
+      <c r="Q32" s="31"/>
+      <c r="R32" s="31"/>
+      <c r="S32" s="31"/>
+      <c r="T32" s="31"/>
+      <c r="U32" s="31"/>
+      <c r="V32" s="31"/>
       <c r="W32" s="7"/>
       <c r="X32" s="7"/>
       <c r="Y32" s="7"/>
@@ -3231,10 +3295,10 @@
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="2"/>
-      <c r="B33" s="28" t="s">
+      <c r="B33" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="37" t="s">
         <v>103</v>
       </c>
       <c r="D33" s="10">
@@ -3252,11 +3316,11 @@
       <c r="H33" s="2">
         <v>0</v>
       </c>
-      <c r="I33" s="22" t="s">
+      <c r="I33" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="J33" s="22"/>
-      <c r="K33" s="22"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
       <c r="L33" s="9" t="s">
         <v>105</v>
       </c>
@@ -3267,16 +3331,16 @@
       </c>
       <c r="P33" s="9"/>
       <c r="Q33" s="9"/>
-      <c r="R33" s="29"/>
-      <c r="S33" s="30"/>
-      <c r="T33" s="30"/>
-      <c r="U33" s="30"/>
-      <c r="V33" s="30"/>
-      <c r="W33" s="30"/>
-      <c r="X33" s="30"/>
-      <c r="Y33" s="30"/>
-      <c r="Z33" s="30"/>
-      <c r="AA33" s="31"/>
+      <c r="R33" s="38"/>
+      <c r="S33" s="39"/>
+      <c r="T33" s="39"/>
+      <c r="U33" s="39"/>
+      <c r="V33" s="39"/>
+      <c r="W33" s="39"/>
+      <c r="X33" s="39"/>
+      <c r="Y33" s="39"/>
+      <c r="Z33" s="39"/>
+      <c r="AA33" s="40"/>
       <c r="AB33" s="8" t="s">
         <v>11</v>
       </c>
@@ -3295,10 +3359,10 @@
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2"/>
-      <c r="B34" s="28" t="s">
+      <c r="B34" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="37" t="s">
         <v>109</v>
       </c>
       <c r="D34" s="10">
@@ -3316,25 +3380,25 @@
       <c r="H34" s="10">
         <v>1</v>
       </c>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="26"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="26"/>
-      <c r="V34" s="26"/>
-      <c r="W34" s="26"/>
-      <c r="X34" s="26"/>
-      <c r="Y34" s="26"/>
-      <c r="Z34" s="26"/>
-      <c r="AA34" s="26"/>
+      <c r="I34" s="35"/>
+      <c r="J34" s="35"/>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
+      <c r="N34" s="35"/>
+      <c r="O34" s="35"/>
+      <c r="P34" s="35"/>
+      <c r="Q34" s="35"/>
+      <c r="R34" s="35"/>
+      <c r="S34" s="35"/>
+      <c r="T34" s="35"/>
+      <c r="U34" s="35"/>
+      <c r="V34" s="35"/>
+      <c r="W34" s="35"/>
+      <c r="X34" s="35"/>
+      <c r="Y34" s="35"/>
+      <c r="Z34" s="35"/>
+      <c r="AA34" s="35"/>
       <c r="AB34" s="8" t="s">
         <v>11</v>
       </c>
@@ -3353,10 +3417,10 @@
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" s="28" t="s">
+      <c r="B35" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="37" t="s">
         <v>112</v>
       </c>
       <c r="D35" s="10">
@@ -3379,22 +3443,22 @@
       </c>
       <c r="J35" s="9"/>
       <c r="K35" s="9"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="25"/>
-      <c r="Q35" s="25"/>
-      <c r="R35" s="25"/>
-      <c r="S35" s="25"/>
-      <c r="T35" s="25"/>
-      <c r="U35" s="25"/>
-      <c r="V35" s="25"/>
-      <c r="W35" s="25"/>
-      <c r="X35" s="25"/>
-      <c r="Y35" s="25"/>
-      <c r="Z35" s="25"/>
-      <c r="AA35" s="25"/>
+      <c r="L35" s="34"/>
+      <c r="M35" s="34"/>
+      <c r="N35" s="34"/>
+      <c r="O35" s="34"/>
+      <c r="P35" s="34"/>
+      <c r="Q35" s="34"/>
+      <c r="R35" s="34"/>
+      <c r="S35" s="34"/>
+      <c r="T35" s="34"/>
+      <c r="U35" s="34"/>
+      <c r="V35" s="34"/>
+      <c r="W35" s="34"/>
+      <c r="X35" s="34"/>
+      <c r="Y35" s="34"/>
+      <c r="Z35" s="34"/>
+      <c r="AA35" s="34"/>
       <c r="AB35" s="8" t="s">
         <v>11</v>
       </c>
@@ -3413,10 +3477,10 @@
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="2"/>
-      <c r="B36" s="28" t="s">
+      <c r="B36" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="37" t="s">
         <v>115</v>
       </c>
       <c r="D36" s="10">
@@ -3439,22 +3503,22 @@
       </c>
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
-      <c r="L36" s="25"/>
-      <c r="M36" s="25"/>
-      <c r="N36" s="25"/>
-      <c r="O36" s="25"/>
-      <c r="P36" s="25"/>
-      <c r="Q36" s="25"/>
-      <c r="R36" s="25"/>
-      <c r="S36" s="25"/>
-      <c r="T36" s="25"/>
-      <c r="U36" s="25"/>
-      <c r="V36" s="25"/>
-      <c r="W36" s="25"/>
-      <c r="X36" s="25"/>
-      <c r="Y36" s="25"/>
-      <c r="Z36" s="25"/>
-      <c r="AA36" s="25"/>
+      <c r="L36" s="34"/>
+      <c r="M36" s="34"/>
+      <c r="N36" s="34"/>
+      <c r="O36" s="34"/>
+      <c r="P36" s="34"/>
+      <c r="Q36" s="34"/>
+      <c r="R36" s="34"/>
+      <c r="S36" s="34"/>
+      <c r="T36" s="34"/>
+      <c r="U36" s="34"/>
+      <c r="V36" s="34"/>
+      <c r="W36" s="34"/>
+      <c r="X36" s="34"/>
+      <c r="Y36" s="34"/>
+      <c r="Z36" s="34"/>
+      <c r="AA36" s="34"/>
       <c r="AB36" s="8" t="s">
         <v>11</v>
       </c>
@@ -3716,25 +3780,25 @@
       <c r="AL46" s="1"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="B47" s="32" t="s">
+      <c r="B47" s="41" t="s">
         <v>117</v>
       </c>
-      <c r="C47" s="33"/>
-      <c r="D47" s="33"/>
-      <c r="E47" s="33"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="33"/>
-      <c r="I47" s="33"/>
-      <c r="J47" s="33"/>
-      <c r="K47" s="33"/>
-      <c r="L47" s="33"/>
-      <c r="M47" s="33"/>
-      <c r="N47" s="33"/>
-      <c r="O47" s="33"/>
-      <c r="P47" s="33"/>
-      <c r="Q47" s="33"/>
-      <c r="R47" s="34"/>
+      <c r="C47" s="42"/>
+      <c r="D47" s="42"/>
+      <c r="E47" s="42"/>
+      <c r="F47" s="42"/>
+      <c r="G47" s="42"/>
+      <c r="H47" s="42"/>
+      <c r="I47" s="42"/>
+      <c r="J47" s="42"/>
+      <c r="K47" s="42"/>
+      <c r="L47" s="42"/>
+      <c r="M47" s="42"/>
+      <c r="N47" s="42"/>
+      <c r="O47" s="42"/>
+      <c r="P47" s="42"/>
+      <c r="Q47" s="42"/>
+      <c r="R47" s="43"/>
       <c r="T47" s="1"/>
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
@@ -3802,10 +3866,10 @@
       <c r="AL48" s="1"/>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="B49" s="35" t="s">
+      <c r="B49" s="44" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="35" t="s">
+      <c r="C49" s="44" t="s">
         <v>121</v>
       </c>
       <c r="D49" s="4" t="s">
@@ -3848,10 +3912,10 @@
       <c r="AL49" s="1"/>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="35" t="s">
+      <c r="B50" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="C50" s="35" t="s">
+      <c r="C50" s="44" t="s">
         <v>125</v>
       </c>
       <c r="D50" s="4" t="s">
@@ -3895,10 +3959,10 @@
       <c r="AL50" s="1"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="B51" s="35" t="s">
+      <c r="B51" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="C51" s="35" t="s">
+      <c r="C51" s="44" t="s">
         <v>129</v>
       </c>
       <c r="D51" s="4" t="s">
@@ -3942,10 +4006,10 @@
       <c r="AL51" s="1"/>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="B52" s="35" t="s">
+      <c r="B52" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="C52" s="35" t="s">
+      <c r="C52" s="44" t="s">
         <v>133</v>
       </c>
       <c r="D52" s="4" t="s">
@@ -3989,10 +4053,10 @@
       <c r="AL52" s="1"/>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="B53" s="35" t="s">
+      <c r="B53" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="C53" s="35" t="s">
+      <c r="C53" s="44" t="s">
         <v>137</v>
       </c>
       <c r="D53" s="4" t="s">
@@ -4546,10 +4610,10 @@
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="36"/>
-      <c r="F67" s="36"/>
-      <c r="G67" s="36"/>
-      <c r="H67" s="36"/>
+      <c r="E67" s="45"/>
+      <c r="F67" s="45"/>
+      <c r="G67" s="45"/>
+      <c r="H67" s="45"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
@@ -4585,10 +4649,10 @@
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="36"/>
-      <c r="F68" s="36"/>
-      <c r="G68" s="36"/>
-      <c r="H68" s="36"/>
+      <c r="E68" s="45"/>
+      <c r="F68" s="45"/>
+      <c r="G68" s="45"/>
+      <c r="H68" s="45"/>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
@@ -4624,10 +4688,10 @@
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
-      <c r="E69" s="36"/>
-      <c r="F69" s="36"/>
-      <c r="G69" s="36"/>
-      <c r="H69" s="36"/>
+      <c r="E69" s="45"/>
+      <c r="F69" s="45"/>
+      <c r="G69" s="45"/>
+      <c r="H69" s="45"/>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
@@ -4663,10 +4727,10 @@
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
-      <c r="E70" s="36"/>
-      <c r="F70" s="36"/>
-      <c r="G70" s="36"/>
-      <c r="H70" s="36"/>
+      <c r="E70" s="45"/>
+      <c r="F70" s="45"/>
+      <c r="G70" s="45"/>
+      <c r="H70" s="45"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
@@ -4702,10 +4766,10 @@
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="36"/>
-      <c r="F71" s="36"/>
-      <c r="G71" s="36"/>
-      <c r="H71" s="36"/>
+      <c r="E71" s="45"/>
+      <c r="F71" s="45"/>
+      <c r="G71" s="45"/>
+      <c r="H71" s="45"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -4741,10 +4805,10 @@
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="36"/>
-      <c r="F72" s="36"/>
-      <c r="G72" s="36"/>
-      <c r="H72" s="36"/>
+      <c r="E72" s="45"/>
+      <c r="F72" s="45"/>
+      <c r="G72" s="45"/>
+      <c r="H72" s="45"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
@@ -4785,7 +4849,7 @@
     <row r="79" ht="15" customHeight="1"/>
     <row r="80" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="114">
+  <mergeCells count="117">
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="L2:S2"/>
     <mergeCell ref="T2:AA2"/>
@@ -4839,13 +4903,16 @@
     <mergeCell ref="R17:AA17"/>
     <mergeCell ref="I18:K18"/>
     <mergeCell ref="L18:N18"/>
-    <mergeCell ref="O18:AA18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="R18:AA18"/>
     <mergeCell ref="I19:K19"/>
     <mergeCell ref="L19:N19"/>
-    <mergeCell ref="O19:AA19"/>
+    <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="R19:AA19"/>
     <mergeCell ref="I20:K20"/>
     <mergeCell ref="L20:N20"/>
-    <mergeCell ref="O20:AA20"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="R20:AA20"/>
     <mergeCell ref="I21:K21"/>
     <mergeCell ref="L21:N21"/>
     <mergeCell ref="O21:Q21"/>

</xml_diff>